<commit_message>
update world cup results
</commit_message>
<xml_diff>
--- a/worldcup_predictions.xlsx
+++ b/worldcup_predictions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\CNE\telegram-bot\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89F229CD-D701-41DE-B45B-DC2B71A4111E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0AF5CC1-DE64-4D4D-83E8-AE905672E5C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="24">
   <si>
     <t>group</t>
   </si>
@@ -91,6 +91,9 @@
   </si>
   <si>
     <t>Scotland</t>
+  </si>
+  <si>
+    <t>Iran</t>
   </si>
 </sst>
 </file>
@@ -859,7 +862,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:A4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.3">
@@ -875,6 +878,11 @@
     <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>21</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update bot and results
</commit_message>
<xml_diff>
--- a/worldcup_predictions.xlsx
+++ b/worldcup_predictions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\CNE\telegram-bot\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF3C2934-DE10-4A29-BC40-53798F236FA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54F61CA1-7779-4675-80C7-FB03F9036A9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="GROUP_STAGE" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="15">
   <si>
     <t>group</t>
   </si>
@@ -67,33 +67,6 @@
   </si>
   <si>
     <t>L</t>
-  </si>
-  <si>
-    <t>Mexico</t>
-  </si>
-  <si>
-    <t>South Korea</t>
-  </si>
-  <si>
-    <t>South Africa</t>
-  </si>
-  <si>
-    <t>Czechia</t>
-  </si>
-  <si>
-    <t>Morocco</t>
-  </si>
-  <si>
-    <t>Haiti</t>
-  </si>
-  <si>
-    <t>Brazil</t>
-  </si>
-  <si>
-    <t>Scotland</t>
-  </si>
-  <si>
-    <t>Iran</t>
   </si>
 </sst>
 </file>
@@ -451,9 +424,6 @@
       <c r="A2" t="s">
         <v>3</v>
       </c>
-      <c r="B2" t="s">
-        <v>15</v>
-      </c>
       <c r="C2">
         <v>1</v>
       </c>
@@ -462,9 +432,6 @@
       <c r="A3" t="s">
         <v>3</v>
       </c>
-      <c r="B3" t="s">
-        <v>16</v>
-      </c>
       <c r="C3">
         <v>2</v>
       </c>
@@ -473,9 +440,6 @@
       <c r="A4" t="s">
         <v>3</v>
       </c>
-      <c r="B4" t="s">
-        <v>17</v>
-      </c>
       <c r="C4">
         <v>3</v>
       </c>
@@ -483,9 +447,6 @@
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>3</v>
-      </c>
-      <c r="B5" t="s">
-        <v>18</v>
       </c>
       <c r="C5">
         <v>4</v>
@@ -527,9 +488,6 @@
       <c r="A10" t="s">
         <v>5</v>
       </c>
-      <c r="B10" t="s">
-        <v>19</v>
-      </c>
       <c r="C10">
         <v>1</v>
       </c>
@@ -538,9 +496,6 @@
       <c r="A11" t="s">
         <v>5</v>
       </c>
-      <c r="B11" t="s">
-        <v>20</v>
-      </c>
       <c r="C11">
         <v>2</v>
       </c>
@@ -549,9 +504,6 @@
       <c r="A12" t="s">
         <v>5</v>
       </c>
-      <c r="B12" t="s">
-        <v>21</v>
-      </c>
       <c r="C12">
         <v>3</v>
       </c>
@@ -559,9 +511,6 @@
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>5</v>
-      </c>
-      <c r="B13" t="s">
-        <v>22</v>
       </c>
       <c r="C13">
         <v>4</v>
@@ -862,27 +811,12 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:A4"/>
+  <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>